<commit_message>
Note donation plan for the 4 duplicate coins in invoice Notes column
</commit_message>
<xml_diff>
--- a/output/invoice_68734_L1019_L1135_FINAL.xlsx
+++ b/output/invoice_68734_L1019_L1135_FINAL.xlsx
@@ -4339,7 +4339,11 @@
       <c r="E124" s="5"/>
       <c r="F124" s="17"/>
       <c r="G124" s="17"/>
-      <c r="H124" s="2"/>
+      <c r="H124" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Duplicate coin - to be donated</t>
+        </is>
+      </c>
       <c r="I124" s="25"/>
       <c r="J124" s="5"/>
       <c r="K124" s="25"/>
@@ -4363,7 +4367,11 @@
       <c r="E125" s="5"/>
       <c r="F125" s="17"/>
       <c r="G125" s="17"/>
-      <c r="H125" s="2"/>
+      <c r="H125" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Duplicate coin - to be donated</t>
+        </is>
+      </c>
       <c r="I125" s="25"/>
       <c r="J125" s="5"/>
       <c r="K125" s="25"/>
@@ -4423,7 +4431,11 @@
       <c r="E127" s="5"/>
       <c r="F127" s="17"/>
       <c r="G127" s="17"/>
-      <c r="H127" s="2"/>
+      <c r="H127" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Duplicate coin - to be donated</t>
+        </is>
+      </c>
       <c r="I127" s="25"/>
       <c r="J127" s="5"/>
       <c r="K127" s="25"/>
@@ -4807,7 +4819,11 @@
       <c r="E138" s="5"/>
       <c r="F138" s="17"/>
       <c r="G138" s="17"/>
-      <c r="H138" s="2"/>
+      <c r="H138" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Duplicate coin - to be donated</t>
+        </is>
+      </c>
       <c r="I138" s="25"/>
       <c r="J138" s="5"/>
       <c r="K138" s="25"/>

</xml_diff>

<commit_message>
Fill Description/Specs/Grade for the 4 duplicate coins in invoice
</commit_message>
<xml_diff>
--- a/output/invoice_68734_L1019_L1135_FINAL.xlsx
+++ b/output/invoice_68734_L1019_L1135_FINAL.xlsx
@@ -4334,9 +4334,21 @@
       <c r="B124" s="17">
         <v>3</v>
       </c>
-      <c r="C124" s="5"/>
-      <c r="D124" s="5"/>
-      <c r="E124" s="5"/>
+      <c r="C124" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Austria (Second Republic). 5 Groschen, 1968. Vienna Mint. Zinc. Austrian eagle type.</t>
+        </is>
+      </c>
+      <c r="D124" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not individually measured</t>
+        </is>
+      </c>
+      <c r="E124" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">VF (photo estimate)</t>
+        </is>
+      </c>
       <c r="F124" s="17"/>
       <c r="G124" s="17"/>
       <c r="H124" s="2" t="inlineStr">
@@ -4362,9 +4374,21 @@
       <c r="B125" s="17">
         <v>4</v>
       </c>
-      <c r="C125" s="5"/>
-      <c r="D125" s="5"/>
-      <c r="E125" s="5"/>
+      <c r="C125" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Austria (Second Republic). 5 Groschen, 1973. Vienna Mint. Zinc. Austrian eagle type.</t>
+        </is>
+      </c>
+      <c r="D125" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not individually measured</t>
+        </is>
+      </c>
+      <c r="E125" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">VF (photo estimate)</t>
+        </is>
+      </c>
       <c r="F125" s="17"/>
       <c r="G125" s="17"/>
       <c r="H125" s="2" t="inlineStr">
@@ -4426,9 +4450,21 @@
       <c r="B127" s="17">
         <v>6</v>
       </c>
-      <c r="C127" s="5"/>
-      <c r="D127" s="5"/>
-      <c r="E127" s="5"/>
+      <c r="C127" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Austria (Second Republic). 5 Groschen, 1966. Vienna Mint. Zinc. Austrian eagle type.</t>
+        </is>
+      </c>
+      <c r="D127" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not individually measured</t>
+        </is>
+      </c>
+      <c r="E127" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">VF (photo estimate)</t>
+        </is>
+      </c>
       <c r="F127" s="17"/>
       <c r="G127" s="17"/>
       <c r="H127" s="2" t="inlineStr">
@@ -4814,9 +4850,21 @@
       <c r="B138" s="17">
         <v>17</v>
       </c>
-      <c r="C138" s="5"/>
-      <c r="D138" s="5"/>
-      <c r="E138" s="5"/>
+      <c r="C138" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Austria (Second Republic). 1 Groschen, 1947. Vienna Mint. Aluminum. Austrian eagle type.</t>
+        </is>
+      </c>
+      <c r="D138" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not individually measured</t>
+        </is>
+      </c>
+      <c r="E138" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">F-VF (photo estimate)</t>
+        </is>
+      </c>
       <c r="F138" s="17"/>
       <c r="G138" s="17"/>
       <c r="H138" s="2" t="inlineStr">

</xml_diff>